<commit_message>
Remove auto-filter buttons from KVP year sheets
https://claude.ai/code/session_0143BHkUCZBxvBT1DPHnv3wk
</commit_message>
<xml_diff>
--- a/KVP_2026.xlsx
+++ b/KVP_2026.xlsx
@@ -17,15 +17,10 @@
   </sheets>
   <definedNames>
     <definedName name="KVPNamenListe">Hilfslisten!$A$2:$A$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026'!$A$4:$I$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'2026'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2025'!$A$4:$I$71</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'2025'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2024'!$A$4:$I$64</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'2024'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'2023'!$A$4:$I$65</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'2023'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'2022'!$A$4:$I$65</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'2022'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2080,7 +2075,6 @@
       <c r="I54" s="47" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I54"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -3551,7 +3545,6 @@
       <c r="I71" s="47" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I71"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -4747,7 +4740,6 @@
       <c r="I64" s="47" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I64"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -5962,7 +5954,6 @@
       <c r="I65" s="47" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I65"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -7175,7 +7166,6 @@
       <c r="I65" s="47" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I65"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>

<commit_message>
KVP Dashboard: 'Top-Thema' durch 'Letzter Eintrag' ersetzt
Die Spalte zeigte sinnlos den ersten Eintrag als 'Top-Thema'.
Jetzt zeigt sie per LOOKUP-Formel den tatsaechlich letzten
(neuesten) Eintrag jedes Jahres an.

https://claude.ai/code/session_0143BHkUCZBxvBT1DPHnv3wk
</commit_message>
<xml_diff>
--- a/KVP_2026.xlsx
+++ b/KVP_2026.xlsx
@@ -878,7 +878,7 @@
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>Top-Thema</t>
+          <t>Letzter Eintrag</t>
         </is>
       </c>
     </row>
@@ -910,7 +910,7 @@
         <v/>
       </c>
       <c r="I8" s="15">
-        <f>IF('2026'!C5&lt;&gt;"",'2026'!C5,"—")</f>
+        <f>IFERROR(LOOKUP(2,1/('2026'!C5:C204&lt;&gt;""),'2026'!C5:C204),"—")</f>
         <v/>
       </c>
     </row>
@@ -942,7 +942,7 @@
         <v/>
       </c>
       <c r="I9" s="23">
-        <f>IF('2025'!C5&lt;&gt;"",'2025'!C5,"—")</f>
+        <f>IFERROR(LOOKUP(2,1/('2025'!C5:C204&lt;&gt;""),'2025'!C5:C204),"—")</f>
         <v/>
       </c>
     </row>
@@ -974,7 +974,7 @@
         <v/>
       </c>
       <c r="I10" s="15">
-        <f>IF('2024'!C5&lt;&gt;"",'2024'!C5,"—")</f>
+        <f>IFERROR(LOOKUP(2,1/('2024'!C5:C204&lt;&gt;""),'2024'!C5:C204),"—")</f>
         <v/>
       </c>
     </row>
@@ -1006,7 +1006,7 @@
         <v/>
       </c>
       <c r="I11" s="23">
-        <f>IF('2023'!C5&lt;&gt;"",'2023'!C5,"—")</f>
+        <f>IFERROR(LOOKUP(2,1/('2023'!C5:C204&lt;&gt;""),'2023'!C5:C204),"—")</f>
         <v/>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
         <v/>
       </c>
       <c r="I12" s="15">
-        <f>IF('2022'!C5&lt;&gt;"",'2022'!C5,"—")</f>
+        <f>IFERROR(LOOKUP(2,1/('2022'!C5:C204&lt;&gt;""),'2022'!C5:C204),"—")</f>
         <v/>
       </c>
     </row>

</xml_diff>